<commit_message>
Use current company identity in inventory reports and enable read-only copying
</commit_message>
<xml_diff>
--- a/tdp_system/templates/inventory_closing_template.xlsx
+++ b/tdp_system/templates/inventory_closing_template.xlsx
@@ -1667,11 +1667,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="171.6" customHeight="1">
-      <c r="A1" s="11" t="inlineStr">
-        <is>
-          <t>CÔNG TY TNHH PHÁT TRIỂN THƯƠNG MẠI THÀNH ĐẠT PHÁT</t>
-        </is>
-      </c>
+      <c r="A1" s="11" t="n"/>
       <c r="B1" s="12" t="n"/>
       <c r="C1" s="12" t="n"/>
       <c r="D1" s="7" t="n"/>
@@ -1679,11 +1675,7 @@
       <c r="I1" s="59" t="n"/>
     </row>
     <row r="2" ht="234" customHeight="1">
-      <c r="A2" s="14" t="inlineStr">
-        <is>
-          <t>Địa chỉ: Số 3/53/33/112A Ngô Quyền, Phường Máy Chai, Quận Ngô Quyền, Thành phố Hải Phòng</t>
-        </is>
-      </c>
+      <c r="A2" s="14" t="n"/>
       <c r="B2" s="12" t="n"/>
       <c r="C2" s="12" t="n"/>
       <c r="D2" s="7" t="n"/>
@@ -1691,11 +1683,7 @@
       <c r="I2" s="57" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="15" t="inlineStr">
-        <is>
-          <t>MST: 0201650135</t>
-        </is>
-      </c>
+      <c r="A3" s="15" t="n"/>
       <c r="B3" s="12" t="n"/>
       <c r="C3" s="12" t="n"/>
       <c r="D3" s="7" t="n"/>

</xml_diff>